<commit_message>
BOM update Changes: - New case - Sockets for relays
</commit_message>
<xml_diff>
--- a/Bill of materials.xlsx
+++ b/Bill of materials.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="77">
   <si>
     <t>Наименование</t>
   </si>
@@ -29,9 +29,6 @@
     <t>Ссылка</t>
   </si>
   <si>
-    <t>RJ45 в корпус</t>
-  </si>
-  <si>
     <t>Назначение</t>
   </si>
   <si>
@@ -92,9 +89,6 @@
     <t>https://www.chipdip.ru/product/hyr-0108-gb-108-bnc-7021-razem-bnc-shteker-zaglushka-hoyutec-18306</t>
   </si>
   <si>
-    <t>Док</t>
-  </si>
-  <si>
     <t>https://www.chipdip.ru/product/bnc-7021-hyr-0108-gb-108-zaglushka-bnc-7021-hyr-0108-ruichi-8007161724</t>
   </si>
   <si>
@@ -102,9 +96,6 @@
   </si>
   <si>
     <t>https://ozon.ru/t/UL99jAh</t>
-  </si>
-  <si>
-    <t>https://lab3dprint.ru/</t>
   </si>
   <si>
     <t>Крепление цепочки должно быть ниже разъема</t>
@@ -173,9 +164,6 @@
     <t>RC0805FR-07100RL</t>
   </si>
   <si>
-    <t>Подключение к прибору для управления</t>
-  </si>
-  <si>
     <t>Надо расположить с противоположной стороны от входного Type-C, там же где коннекторы</t>
   </si>
   <si>
@@ -217,18 +205,6 @@
 Надо проверить соответствие высоты резьбы на плате с 3D-моделью</t>
   </si>
   <si>
-    <t>https://www.chipdip.ru/product/15-6-170x130x55-korpus-dlya-rea-plastikovyy-ruichi-8007169529</t>
-  </si>
-  <si>
-    <t>RUICHI 15-6</t>
-  </si>
-  <si>
-    <t>Возможно лучше напечатать</t>
-  </si>
-  <si>
-    <t>Корпус 170x130x55 мм</t>
-  </si>
-  <si>
     <t>https://ozon.ru/t/quQb2ul</t>
   </si>
   <si>
@@ -239,6 +215,42 @@
   </si>
   <si>
     <t>Резисторы 100 кОм</t>
+  </si>
+  <si>
+    <t>https://aliexpress.ru/item/1005009317440293.html</t>
+  </si>
+  <si>
+    <t>DIP 4 IC SOCKET</t>
+  </si>
+  <si>
+    <t>DIP-4 панельки для установки реле</t>
+  </si>
+  <si>
+    <t>по 2 шт на 1 реле</t>
+  </si>
+  <si>
+    <t>В наличии</t>
+  </si>
+  <si>
+    <t>G733</t>
+  </si>
+  <si>
+    <t>Корпус 260x180x105 мм</t>
+  </si>
+  <si>
+    <t>https://www.chipdip.ru/product/g733-korpus-dlya-rea-260x180x105mm-plastik-gainta-236156751</t>
+  </si>
+  <si>
+    <t>https://static.chipdip.ru/lib/414/DOC014414780.pdf</t>
+  </si>
+  <si>
+    <t>Подключение к прибору</t>
+  </si>
+  <si>
+    <t>RJ45 на корпус</t>
+  </si>
+  <si>
+    <t>Документация</t>
   </si>
 </sst>
 </file>
@@ -262,12 +274,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -298,7 +316,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -309,23 +327,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -629,13 +641,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" style="1" bestFit="1" customWidth="1"/>
@@ -652,36 +664,36 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="9" t="s">
-        <v>38</v>
+      <c r="I1" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -693,47 +705,47 @@
         <v>10600</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2">
         <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F3" s="2">
         <v>300</v>
       </c>
       <c r="G3" s="2">
-        <f t="shared" ref="G3:G10" si="0">B3*F3</f>
+        <f t="shared" ref="G3:G11" si="0">B3*F3</f>
         <v>4800</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2">
         <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -745,23 +757,23 @@
         <v>176</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F5" s="2">
         <v>2</v>
@@ -771,21 +783,21 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2">
@@ -793,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I6" s="2"/>
     </row>
@@ -801,11 +813,11 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -814,17 +826,17 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2">
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F8" s="2">
         <v>42</v>
@@ -834,23 +846,23 @@
         <v>84</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F9" s="2">
         <v>110</v>
@@ -860,23 +872,23 @@
         <v>220</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F10" s="2">
         <v>45</v>
@@ -886,11 +898,40 @@
         <v>360</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>63</v>
-      </c>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="2">
+        <f>B3*2</f>
+        <v>32</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -909,7 +950,7 @@
     <col min="5" max="5" width="51" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="96.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="96.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="99" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -922,51 +963,51 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>25</v>
+      <c r="I1" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2"/>
-      <c r="E2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2">
+        <v>1660</v>
+      </c>
       <c r="G2" s="2">
         <f t="shared" ref="G2:G5" si="0">F2*B2</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>65</v>
+        <v>1660</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -977,11 +1018,11 @@
         <v>8</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F3" s="2">
         <v>140</v>
@@ -990,26 +1031,26 @@
         <f t="shared" si="0"/>
         <v>1120</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="B4" s="2">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F4" s="2">
         <v>1470</v>
@@ -1018,26 +1059,26 @@
         <f t="shared" si="0"/>
         <v>1470</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>27</v>
+      <c r="H4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="F5" s="2">
         <v>213</v>
@@ -1046,23 +1087,24 @@
         <f t="shared" si="0"/>
         <v>213</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>69</v>
-      </c>
+      <c r="H5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2">
         <v>1</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" s="2">
         <v>146</v>
@@ -1071,23 +1113,24 @@
         <f>F6*B6</f>
         <v>146</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>13</v>
-      </c>
+      <c r="H6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7" s="2">
         <v>211</v>
@@ -1096,23 +1139,26 @@
         <f t="shared" ref="G7:G8" si="1">F7*B7</f>
         <v>211</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>28</v>
-      </c>
+      <c r="H7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>69</v>
+      </c>
       <c r="E8" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F8" s="2">
         <v>63</v>
@@ -1121,9 +1167,10 @@
         <f t="shared" si="1"/>
         <v>63</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>17</v>
-      </c>
+      <c r="H8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1134,7 +1181,7 @@
     <hyperlink ref="I4" r:id="rId5"/>
     <hyperlink ref="H7" r:id="rId6"/>
     <hyperlink ref="H8" r:id="rId7"/>
-    <hyperlink ref="H2" r:id="rId8"/>
+    <hyperlink ref="I2" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>

</xml_diff>

<commit_message>
Add BomDoc and update excel-based BOM
</commit_message>
<xml_diff>
--- a/Bill of materials.xlsx
+++ b/Bill of materials.xlsx
@@ -8,14 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Плата" sheetId="1" r:id="rId1"/>
-    <sheet name="Конструктив" sheetId="3" r:id="rId2"/>
+    <sheet name="Прочее" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="81">
   <si>
     <t>Наименование</t>
   </si>
@@ -120,9 +120,6 @@
   </si>
   <si>
     <t>https://www.chipdip.ru/product/irlml2803trpbf-tranzistor-n-kanal-30v-1.2a-logic-infineon-447047429</t>
-  </si>
-  <si>
-    <t>Аналоги</t>
   </si>
   <si>
     <t>Полный аналог
@@ -214,9 +211,6 @@
     <t>Тонкий короткий провод, угловой для удобства</t>
   </si>
   <si>
-    <t>Резисторы 100 кОм</t>
-  </si>
-  <si>
     <t>https://aliexpress.ru/item/1005009317440293.html</t>
   </si>
   <si>
@@ -251,6 +245,24 @@
   </si>
   <si>
     <t>Документация</t>
+  </si>
+  <si>
+    <t>RC0805FR-07100KL</t>
+  </si>
+  <si>
+    <t>Резисторы 10 кОм</t>
+  </si>
+  <si>
+    <t>https://www.chipdip.ru/product/0.125vt-0805-10-kom-1-rc0805fr-0710kl-chip-rezistor-yageo-9000272499</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>Не требуется</t>
+  </si>
+  <si>
+    <t>Требуется</t>
   </si>
 </sst>
 </file>
@@ -274,7 +286,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -284,6 +296,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -316,7 +346,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -327,9 +357,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -338,6 +365,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -647,43 +683,41 @@
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="97.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="97.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="44.28515625" style="1" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="I1" s="9"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -693,9 +727,11 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="2"/>
+        <v>36</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2">
         <v>10600</v>
@@ -717,11 +753,13 @@
         <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="F3" s="2">
         <v>300</v>
@@ -734,7 +772,7 @@
         <v>30</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -747,8 +785,12 @@
       <c r="C4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="D4" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="F4" s="2">
         <v>11</v>
       </c>
@@ -760,83 +802,108 @@
         <v>34</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="2"/>
+        <v>39</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E5" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F5" s="2">
         <v>2</v>
       </c>
       <c r="G5" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="2"/>
+        <v>46</v>
+      </c>
+      <c r="B6" s="2">
+        <v>16</v>
+      </c>
       <c r="C6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" s="2"/>
+      <c r="F6" s="2">
+        <v>2</v>
+      </c>
       <c r="G6" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="2">
+        <v>16</v>
+      </c>
       <c r="C7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="F7" s="2">
+        <v>2</v>
+      </c>
+      <c r="G7" s="2">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B8" s="2">
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>79</v>
+      </c>
       <c r="E8" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F8" s="2">
         <v>42</v>
@@ -846,23 +913,25 @@
         <v>84</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E9" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F9" s="2">
         <v>110</v>
@@ -872,23 +941,25 @@
         <v>220</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E10" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10" s="2">
         <v>45</v>
@@ -898,28 +969,28 @@
         <v>360</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B11" s="2">
         <f>B3*2</f>
         <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>69</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -929,12 +1000,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -956,45 +1028,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>76</v>
+      <c r="I1" s="9" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2">
         <v>1660</v>
@@ -1003,11 +1077,11 @@
         <f t="shared" ref="G2:G5" si="0">F2*B2</f>
         <v>1660</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>73</v>
+      <c r="H2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1020,7 +1094,9 @@
       <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="7" t="s">
+        <v>79</v>
+      </c>
       <c r="E3" s="2" t="s">
         <v>27</v>
       </c>
@@ -1031,22 +1107,22 @@
         <f t="shared" si="0"/>
         <v>1120</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B4" s="2">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
@@ -1059,16 +1135,16 @@
         <f t="shared" si="0"/>
         <v>1470</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
@@ -1078,7 +1154,7 @@
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F5" s="2">
         <v>213</v>
@@ -1087,8 +1163,8 @@
         <f t="shared" si="0"/>
         <v>213</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>61</v>
+      <c r="H5" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1113,7 +1189,7 @@
         <f>F6*B6</f>
         <v>146</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I6" s="2"/>
@@ -1139,7 +1215,7 @@
         <f t="shared" ref="G7:G8" si="1">F7*B7</f>
         <v>211</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="5" t="s">
         <v>26</v>
       </c>
       <c r="I7" s="2"/>
@@ -1154,11 +1230,11 @@
       <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>69</v>
+      <c r="D8" s="4" t="s">
+        <v>67</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F8" s="2">
         <v>63</v>
@@ -1167,7 +1243,7 @@
         <f t="shared" si="1"/>
         <v>63</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I8" s="2"/>

</xml_diff>